<commit_message>
use real validation_methods.xlsx in AP fixtures; switch event to IFRS New RFD / V900W
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/fip_ZQ9_VALMSG.xlsx
+++ b/test_data/fixtures/fip_ZQ9_VALMSG.xlsx
@@ -476,12 +476,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>V900A</t>
+          <t>V900W</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Test method</t>
+          <t>Warning method</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -528,12 +528,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>V900A</t>
+          <t>V900W</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Test method</t>
+          <t>Warning method</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">

</xml_diff>